<commit_message>
Training database faculty improved
</commit_message>
<xml_diff>
--- a/backend/Training Calendar 2025-26 Final.xlsx
+++ b/backend/Training Calendar 2025-26 Final.xlsx
@@ -1,22 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\siddh_2eavk38\IRDT_Training_Portal\backend\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35125434-C06F-4E8C-A4AF-A0F7D204BA03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{89CADDD2-9C76-4066-AC55-BAE39053FDCC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Training Calendar 2025-26" sheetId="1" r:id="rId1"/>
     <sheet name="Data" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="145621"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -63,9 +57,6 @@
     <t>End Date</t>
   </si>
   <si>
-    <t>Faculy</t>
-  </si>
-  <si>
     <t>No.</t>
   </si>
   <si>
@@ -93,9 +84,6 @@
     <t>25-Apr-25</t>
   </si>
   <si>
-    <t>KMS</t>
-  </si>
-  <si>
     <t>ICT-2</t>
   </si>
   <si>
@@ -111,9 +99,6 @@
     <t>Online</t>
   </si>
   <si>
-    <t>GKK</t>
-  </si>
-  <si>
     <t>IRDT 2</t>
   </si>
   <si>
@@ -124,9 +109,6 @@
   </si>
   <si>
     <t>30-May-25</t>
-  </si>
-  <si>
-    <t>APS</t>
   </si>
   <si>
     <t>ME-5</t>
@@ -139,9 +121,6 @@
     <t>Workshop Instructors from Mechanical Branch</t>
   </si>
   <si>
-    <t>SL</t>
-  </si>
-  <si>
     <t>IRDT 3</t>
   </si>
   <si>
@@ -296,9 +275,6 @@
   </si>
   <si>
     <t>Faculty of Computer, Electronics and allied Engineering disciplines</t>
-  </si>
-  <si>
-    <t>VK</t>
   </si>
   <si>
     <t>ESTC 1</t>
@@ -934,13 +910,31 @@
   </si>
   <si>
     <t>Training Type</t>
+  </si>
+  <si>
+    <t>Kunwer Mrityunjay Singh</t>
+  </si>
+  <si>
+    <t>Atma Prakash Singh</t>
+  </si>
+  <si>
+    <t>Shyam Lal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vikas Kulshreshth </t>
+  </si>
+  <si>
+    <t>Gaurav Kishor Kanaujia</t>
+  </si>
+  <si>
+    <t>Faculty</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1355,7 +1349,6 @@
         <sz val="13"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1386,7 +1379,6 @@
         <sz val="13"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1417,7 +1409,6 @@
         <sz val="13"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1448,7 +1439,6 @@
         <sz val="13"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1479,7 +1469,6 @@
         <sz val="13"/>
         <color auto="1"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1510,7 +1499,6 @@
         <sz val="13"/>
         <color auto="1"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1541,7 +1529,6 @@
         <sz val="13"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1572,7 +1559,6 @@
         <sz val="13"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1603,7 +1589,6 @@
         <sz val="13"/>
         <color rgb="FF000000"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1634,7 +1619,6 @@
         <sz val="13"/>
         <color rgb="FF000000"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1665,7 +1649,6 @@
         <sz val="13"/>
         <color rgb="FF000000"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1696,7 +1679,6 @@
         <sz val="13"/>
         <color rgb="FF000000"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1727,7 +1709,6 @@
         <sz val="13"/>
         <color theme="1"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1751,7 +1732,6 @@
         <vertAlign val="baseline"/>
         <sz val="13"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1779,7 +1759,6 @@
         <vertAlign val="baseline"/>
         <sz val="13"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1807,7 +1786,6 @@
         <vertAlign val="baseline"/>
         <sz val="13"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1835,7 +1813,6 @@
         <vertAlign val="baseline"/>
         <sz val="13"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1868,7 +1845,6 @@
         <sz val="13"/>
         <color auto="1"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -1907,7 +1883,6 @@
         <sz val="13"/>
         <color auto="1"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -1941,7 +1916,6 @@
         <vertAlign val="baseline"/>
         <sz val="13"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1969,7 +1943,6 @@
         <vertAlign val="baseline"/>
         <sz val="13"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2002,7 +1975,6 @@
         <sz val="13"/>
         <color rgb="FF000000"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2035,7 +2007,6 @@
         <sz val="13"/>
         <color rgb="FF000000"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2068,7 +2039,6 @@
         <sz val="13"/>
         <color rgb="FF000000"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2101,7 +2071,6 @@
         <sz val="13"/>
         <color rgb="FF000000"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2129,7 +2098,6 @@
         <vertAlign val="baseline"/>
         <sz val="13"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2162,7 +2130,6 @@
         <vertAlign val="baseline"/>
         <sz val="13"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2192,7 +2159,6 @@
         <vertAlign val="baseline"/>
         <sz val="13"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2218,7 +2184,6 @@
         <sz val="13"/>
         <color auto="1"/>
         <name val="Times New Roman"/>
-        <family val="1"/>
         <scheme val="none"/>
       </font>
       <fill>
@@ -2253,22 +2218,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0F8807A6-DC54-42FE-AABF-12EF895565BA}" name="Table658" displayName="Table658" ref="A1:M94" totalsRowCount="1" headerRowDxfId="31" dataDxfId="29" totalsRowDxfId="27" headerRowBorderDxfId="30" tableBorderDxfId="28" totalsRowBorderDxfId="26">
-  <autoFilter ref="A1:M93" xr:uid="{0F8807A6-DC54-42FE-AABF-12EF895565BA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table658" displayName="Table658" ref="A1:M94" totalsRowCount="1" headerRowDxfId="31" dataDxfId="29" totalsRowDxfId="27" headerRowBorderDxfId="30" tableBorderDxfId="28" totalsRowBorderDxfId="26">
+  <autoFilter ref="A1:M93"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{7D1BAA6A-C6D0-4F48-B2FF-E2212ED1927F}" name="Sr.No" dataDxfId="25" totalsRowDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{E893E372-730E-4E92-89E6-736EE2DAEFF6}" name="Code" dataDxfId="24" totalsRowDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{6AD30E5F-8C90-465E-BEE4-17904C8FE3FA}" name="Name of Programme" dataDxfId="23" totalsRowDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{01973A88-9E22-4901-94EC-2DC1FD586F57}" name="Target Group" dataDxfId="22" totalsRowDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{3DD04297-B53D-4EDC-B0FC-DD166F1FA567}" name="Venue" dataDxfId="21" totalsRowDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{C053BA59-964A-4E39-BB21-43F1A7A28B75}" name="Mode" dataDxfId="20" totalsRowDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{C1C732F6-E7C4-4DFE-8574-B867795B165C}" name="Training Type" dataDxfId="19" totalsRowDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{86643A26-8B05-419F-B888-32FFE27BE100}" name="Start Date" dataDxfId="18" totalsRowDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{ABAA7C77-2335-4C73-A1D3-AE0225A9230B}" name="End Date" dataDxfId="17" totalsRowDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{C8526EBA-F35A-45DE-8D0E-D699137D6CC4}" name="Faculy" dataDxfId="16" totalsRowDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{0767DE1D-C39F-453F-9DDF-F0B0F6657270}" name="No." totalsRowFunction="sum" dataDxfId="15" totalsRowDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{6A4BA237-A6F7-4B4A-84DF-E6784C20A405}" name="Remark" dataDxfId="14" totalsRowDxfId="1"/>
-    <tableColumn id="13" xr3:uid="{1911C9CC-1176-4BC9-978E-1B3543DF58C0}" name="Status" dataDxfId="13" totalsRowDxfId="0"/>
+    <tableColumn id="1" name="Sr.No" dataDxfId="25" totalsRowDxfId="12"/>
+    <tableColumn id="2" name="Code" dataDxfId="24" totalsRowDxfId="11"/>
+    <tableColumn id="3" name="Name of Programme" dataDxfId="23" totalsRowDxfId="10"/>
+    <tableColumn id="4" name="Target Group" dataDxfId="22" totalsRowDxfId="9"/>
+    <tableColumn id="5" name="Venue" dataDxfId="21" totalsRowDxfId="8"/>
+    <tableColumn id="6" name="Mode" dataDxfId="20" totalsRowDxfId="7"/>
+    <tableColumn id="7" name="Training Type" dataDxfId="19" totalsRowDxfId="6"/>
+    <tableColumn id="8" name="Start Date" dataDxfId="18" totalsRowDxfId="5"/>
+    <tableColumn id="9" name="End Date" dataDxfId="17" totalsRowDxfId="4"/>
+    <tableColumn id="10" name="Faculty" dataDxfId="16" totalsRowDxfId="3"/>
+    <tableColumn id="11" name="No." totalsRowFunction="sum" dataDxfId="15" totalsRowDxfId="2"/>
+    <tableColumn id="12" name="Remark" dataDxfId="14" totalsRowDxfId="1"/>
+    <tableColumn id="13" name="Status" dataDxfId="13" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2317,7 +2282,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -2369,7 +2334,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -2583,34 +2548,34 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21989BAB-43E9-4453-978E-88EFE49FDD3D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M94"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="6.42578125" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.28515625" style="31" customWidth="1"/>
-    <col min="4" max="4" width="32.7109375" style="31" customWidth="1"/>
-    <col min="5" max="5" width="14.28515625" style="31" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.375" customWidth="1"/>
+    <col min="2" max="2" width="9.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.25" style="31" customWidth="1"/>
+    <col min="4" max="4" width="32.75" style="31" customWidth="1"/>
+    <col min="5" max="5" width="14.25" style="31" customWidth="1"/>
+    <col min="6" max="6" width="10.25" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8" customWidth="1"/>
-    <col min="8" max="8" width="13.28515625" customWidth="1"/>
-    <col min="9" max="9" width="12.42578125" customWidth="1"/>
-    <col min="10" max="10" width="8.42578125" customWidth="1"/>
-    <col min="11" max="11" width="6.42578125" customWidth="1"/>
+    <col min="8" max="8" width="13.25" customWidth="1"/>
+    <col min="9" max="9" width="12.375" customWidth="1"/>
+    <col min="10" max="10" width="39.5" customWidth="1"/>
+    <col min="11" max="11" width="6.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="16.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2630,7 +2595,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>6</v>
@@ -2639,19 +2604,19 @@
         <v>7</v>
       </c>
       <c r="J1" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="L1" s="4" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="16.5">
       <c r="A2" s="5"/>
       <c r="B2" s="6"/>
       <c r="C2" s="7"/>
@@ -2668,75 +2633,75 @@
       <c r="L2" s="32"/>
       <c r="M2" s="32"/>
     </row>
-    <row r="3" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="33">
       <c r="A3" s="10">
         <v>1</v>
       </c>
       <c r="B3" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="D3" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="E3" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="14" t="s">
-        <v>13</v>
-      </c>
       <c r="F3" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G3" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="I3" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="13" t="s">
-        <v>17</v>
-      </c>
       <c r="J3" s="11" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K3" s="11">
         <v>40</v>
       </c>
       <c r="L3" s="11" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="M3" s="11"/>
     </row>
-    <row r="4" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="33">
       <c r="A4" s="10">
         <v>2</v>
       </c>
       <c r="B4" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="E4" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="F4" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>23</v>
-      </c>
       <c r="G4" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="I4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="13" t="s">
-        <v>17</v>
-      </c>
       <c r="J4" s="11" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K4" s="11">
         <v>15</v>
@@ -2744,7 +2709,7 @@
       <c r="L4" s="11"/>
       <c r="M4" s="11"/>
     </row>
-    <row r="5" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="16.5">
       <c r="A5" s="15"/>
       <c r="B5" s="6"/>
       <c r="C5" s="7"/>
@@ -2761,75 +2726,75 @@
       <c r="L5" s="16"/>
       <c r="M5" s="16"/>
     </row>
-    <row r="6" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="33">
       <c r="A6" s="10">
         <v>3</v>
       </c>
       <c r="B6" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6" s="13" t="s">
-        <v>28</v>
-      </c>
       <c r="J6" s="11" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K6" s="11">
         <v>40</v>
       </c>
       <c r="L6" s="11" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="M6" s="11"/>
     </row>
-    <row r="7" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="33">
       <c r="A7" s="10">
         <v>4</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H7" s="13" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K7" s="11">
         <v>15</v>
@@ -2837,7 +2802,7 @@
       <c r="L7" s="11"/>
       <c r="M7" s="11"/>
     </row>
-    <row r="8" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="16.5">
       <c r="A8" s="15"/>
       <c r="B8" s="6"/>
       <c r="C8" s="18"/>
@@ -2854,36 +2819,36 @@
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
     </row>
-    <row r="9" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="33">
       <c r="A9" s="15">
         <v>5</v>
       </c>
       <c r="B9" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="I9" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="H9" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="I9" s="17" t="s">
-        <v>39</v>
-      </c>
       <c r="J9" s="16" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K9" s="16">
         <v>40</v>
@@ -2891,75 +2856,75 @@
       <c r="L9" s="16"/>
       <c r="M9" s="16"/>
     </row>
-    <row r="10" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="33">
       <c r="A10" s="10">
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="D10" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="14" t="s">
-        <v>13</v>
-      </c>
       <c r="F10" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="J10" s="11" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K10" s="11">
         <v>40</v>
       </c>
       <c r="L10" s="11" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="M10" s="11"/>
     </row>
-    <row r="11" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="33">
       <c r="A11" s="10">
         <v>7</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H11" s="13" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="J11" s="11" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K11" s="11">
         <v>15</v>
@@ -2967,36 +2932,36 @@
       <c r="L11" s="11"/>
       <c r="M11" s="11"/>
     </row>
-    <row r="12" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="33">
       <c r="A12" s="15">
         <v>8</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="I12" s="17" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="J12" s="16" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K12" s="16">
         <v>15</v>
@@ -3004,36 +2969,36 @@
       <c r="L12" s="16"/>
       <c r="M12" s="16"/>
     </row>
-    <row r="13" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" ht="49.5">
       <c r="A13" s="15">
         <v>9</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="I13" s="17" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="J13" s="16" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K13" s="16">
         <v>20</v>
@@ -3041,36 +3006,36 @@
       <c r="L13" s="16"/>
       <c r="M13" s="16"/>
     </row>
-    <row r="14" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="33">
       <c r="A14" s="15">
         <v>10</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="I14" s="17" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="J14" s="16" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K14" s="16">
         <v>40</v>
@@ -3078,75 +3043,75 @@
       <c r="L14" s="16"/>
       <c r="M14" s="16"/>
     </row>
-    <row r="15" spans="1:13" ht="66" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="49.5">
       <c r="A15" s="10">
         <v>11</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H15" s="13" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K15" s="11">
         <v>40</v>
       </c>
       <c r="L15" s="11" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="M15" s="11"/>
     </row>
-    <row r="16" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="16.5">
       <c r="A16" s="15">
         <v>12</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="I16" s="17" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="J16" s="16" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K16" s="16">
         <v>35</v>
@@ -3154,36 +3119,36 @@
       <c r="L16" s="16"/>
       <c r="M16" s="16"/>
     </row>
-    <row r="17" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" ht="33">
       <c r="A17" s="15">
         <v>13</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H17" s="17" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="I17" s="17" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="J17" s="16" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K17" s="16">
         <v>40</v>
@@ -3191,7 +3156,7 @@
       <c r="L17" s="16"/>
       <c r="M17" s="16"/>
     </row>
-    <row r="18" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" ht="16.5">
       <c r="A18" s="15"/>
       <c r="B18" s="6"/>
       <c r="C18" s="7"/>
@@ -3208,27 +3173,27 @@
       <c r="L18" s="16"/>
       <c r="M18" s="16"/>
     </row>
-    <row r="19" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="33">
       <c r="A19" s="10">
         <v>14</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H19" s="19">
         <v>45845</v>
@@ -3237,37 +3202,37 @@
         <v>45849</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K19" s="11">
         <v>30</v>
       </c>
       <c r="L19" s="11"/>
       <c r="M19" s="11" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="33">
       <c r="A20" s="10">
         <v>15</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H20" s="19">
         <v>45845</v>
@@ -3276,7 +3241,7 @@
         <v>45849</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K20" s="11">
         <v>15</v>
@@ -3284,27 +3249,27 @@
       <c r="L20" s="11"/>
       <c r="M20" s="11"/>
     </row>
-    <row r="21" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" ht="33">
       <c r="A21" s="10">
         <v>16</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H21" s="19">
         <v>45845</v>
@@ -3313,7 +3278,7 @@
         <v>45849</v>
       </c>
       <c r="J21" s="11" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K21" s="11">
         <v>15</v>
@@ -3321,36 +3286,36 @@
       <c r="L21" s="11"/>
       <c r="M21" s="11"/>
     </row>
-    <row r="22" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" ht="16.5">
       <c r="A22" s="15">
         <v>17</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H22" s="17" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="I22" s="17" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="J22" s="16" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K22" s="16">
         <v>35</v>
@@ -3358,36 +3323,36 @@
       <c r="L22" s="16"/>
       <c r="M22" s="16"/>
     </row>
-    <row r="23" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" ht="33">
       <c r="A23" s="15">
         <v>18</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H23" s="17" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="I23" s="17" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="J23" s="16" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K23" s="16">
         <v>35</v>
@@ -3395,114 +3360,114 @@
       <c r="L23" s="16"/>
       <c r="M23" s="16"/>
     </row>
-    <row r="24" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" ht="49.5">
       <c r="A24" s="10">
         <v>19</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H24" s="13" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="J24" s="11" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K24" s="11">
         <v>15</v>
       </c>
       <c r="L24" s="11"/>
       <c r="M24" s="11" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" ht="66" x14ac:dyDescent="0.25">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="49.5">
       <c r="A25" s="15">
         <v>20</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F25" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H25" s="17" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="I25" s="17" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="J25" s="16" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K25" s="16">
         <v>40</v>
       </c>
       <c r="L25" s="16" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="M25" s="16"/>
     </row>
-    <row r="26" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" ht="33">
       <c r="A26" s="15">
         <v>21</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F26" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H26" s="17" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="I26" s="17" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="J26" s="16" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K26" s="16">
         <v>35</v>
@@ -3510,36 +3475,36 @@
       <c r="L26" s="16"/>
       <c r="M26" s="16"/>
     </row>
-    <row r="27" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" ht="33">
       <c r="A27" s="15">
         <v>22</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F27" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H27" s="17" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="I27" s="17" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="J27" s="16" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K27" s="16">
         <v>40</v>
@@ -3547,36 +3512,36 @@
       <c r="L27" s="16"/>
       <c r="M27" s="16"/>
     </row>
-    <row r="28" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" ht="33">
       <c r="A28" s="15">
         <v>23</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F28" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G28" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H28" s="17" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="I28" s="17" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="J28" s="16" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K28" s="16">
         <v>35</v>
@@ -3584,7 +3549,7 @@
       <c r="L28" s="16"/>
       <c r="M28" s="16"/>
     </row>
-    <row r="29" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" ht="16.5">
       <c r="A29" s="15"/>
       <c r="B29" s="6"/>
       <c r="C29" s="7"/>
@@ -3601,27 +3566,27 @@
       <c r="L29" s="16"/>
       <c r="M29" s="16"/>
     </row>
-    <row r="30" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" ht="16.5">
       <c r="A30" s="10">
         <v>24</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H30" s="19">
         <v>45873</v>
@@ -3630,37 +3595,37 @@
         <v>45877</v>
       </c>
       <c r="J30" s="11" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K30" s="11">
         <v>30</v>
       </c>
       <c r="L30" s="11"/>
       <c r="M30" s="11" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" ht="33">
       <c r="A31" s="10">
         <v>25</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G31" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H31" s="19">
         <v>45873</v>
@@ -3669,7 +3634,7 @@
         <v>45877</v>
       </c>
       <c r="J31" s="11" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K31" s="11">
         <v>15</v>
@@ -3677,27 +3642,27 @@
       <c r="L31" s="11"/>
       <c r="M31" s="11"/>
     </row>
-    <row r="32" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" ht="33">
       <c r="A32" s="10">
         <v>26</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D32" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E32" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F32" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E32" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="F32" s="11" t="s">
-        <v>23</v>
-      </c>
       <c r="G32" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H32" s="19">
         <v>45873</v>
@@ -3706,7 +3671,7 @@
         <v>45877</v>
       </c>
       <c r="J32" s="11" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K32" s="11">
         <v>15</v>
@@ -3714,27 +3679,27 @@
       <c r="L32" s="11"/>
       <c r="M32" s="11"/>
     </row>
-    <row r="33" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" ht="33">
       <c r="A33" s="10">
         <v>27</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G33" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H33" s="19">
         <v>45873</v>
@@ -3743,7 +3708,7 @@
         <v>45877</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K33" s="11">
         <v>35</v>
@@ -3751,27 +3716,27 @@
       <c r="L33" s="11"/>
       <c r="M33" s="11"/>
     </row>
-    <row r="34" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" ht="33">
       <c r="A34" s="10">
         <v>28</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H34" s="19">
         <v>45873</v>
@@ -3780,7 +3745,7 @@
         <v>45877</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K34" s="11">
         <v>40</v>
@@ -3788,36 +3753,36 @@
       <c r="L34" s="11"/>
       <c r="M34" s="11"/>
     </row>
-    <row r="35" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" ht="33">
       <c r="A35" s="15">
         <v>29</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="C35" s="18" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F35" s="16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H35" s="17" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="I35" s="17" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="J35" s="16" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K35" s="16">
         <v>15</v>
@@ -3825,36 +3790,36 @@
       <c r="L35" s="16"/>
       <c r="M35" s="16"/>
     </row>
-    <row r="36" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" ht="16.5">
       <c r="A36" s="15">
         <v>30</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D36" s="18" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F36" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G36" s="16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H36" s="17" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="I36" s="17" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="J36" s="16" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K36" s="16">
         <v>35</v>
@@ -3862,7 +3827,7 @@
       <c r="L36" s="16"/>
       <c r="M36" s="16"/>
     </row>
-    <row r="37" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" ht="16.5">
       <c r="A37" s="15"/>
       <c r="B37" s="6"/>
       <c r="C37" s="7"/>
@@ -3879,75 +3844,75 @@
       <c r="L37" s="16"/>
       <c r="M37" s="16"/>
     </row>
-    <row r="38" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" ht="33">
       <c r="A38" s="10">
         <v>31</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="D38" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E38" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="E38" s="14" t="s">
-        <v>13</v>
-      </c>
       <c r="F38" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H38" s="13" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="I38" s="13" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="J38" s="11" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K38" s="11">
         <v>40</v>
       </c>
       <c r="L38" s="11" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="M38" s="11"/>
     </row>
-    <row r="39" spans="1:13" ht="66" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" ht="49.5">
       <c r="A39" s="10">
         <v>32</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H39" s="13" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="I39" s="13" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="J39" s="11" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K39" s="11">
         <v>40</v>
@@ -3955,36 +3920,36 @@
       <c r="L39" s="11"/>
       <c r="M39" s="11"/>
     </row>
-    <row r="40" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" ht="33">
       <c r="A40" s="10">
         <v>33</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="F40" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G40" s="11" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H40" s="13" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="I40" s="13" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="J40" s="11" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K40" s="11">
         <v>35</v>
@@ -3992,36 +3957,36 @@
       <c r="L40" s="11"/>
       <c r="M40" s="11"/>
     </row>
-    <row r="41" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" ht="49.5">
       <c r="A41" s="10">
         <v>34</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G41" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H41" s="13" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="I41" s="13" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="J41" s="11" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K41" s="11">
         <v>15</v>
@@ -4029,75 +3994,75 @@
       <c r="L41" s="11"/>
       <c r="M41" s="11"/>
     </row>
-    <row r="42" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" ht="33">
       <c r="A42" s="15">
         <v>35</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="E42" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G42" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H42" s="17" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="I42" s="17" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="J42" s="16" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K42" s="16">
         <v>20</v>
       </c>
       <c r="L42" s="16"/>
       <c r="M42" s="16" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" ht="33">
       <c r="A43" s="15">
         <v>36</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F43" s="16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H43" s="17" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="I43" s="17" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="J43" s="16" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K43" s="16">
         <v>15</v>
@@ -4105,36 +4070,36 @@
       <c r="L43" s="16"/>
       <c r="M43" s="16"/>
     </row>
-    <row r="44" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" ht="33">
       <c r="A44" s="15">
         <v>37</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C44" s="18" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E44" s="18" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H44" s="17" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="I44" s="17" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="J44" s="16" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K44" s="16">
         <v>15</v>
@@ -4142,36 +4107,36 @@
       <c r="L44" s="16"/>
       <c r="M44" s="16"/>
     </row>
-    <row r="45" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" ht="33">
       <c r="A45" s="15">
         <v>38</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H45" s="17" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="I45" s="17" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="J45" s="16" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K45" s="16">
         <v>35</v>
@@ -4179,36 +4144,36 @@
       <c r="L45" s="16"/>
       <c r="M45" s="16"/>
     </row>
-    <row r="46" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" ht="33">
       <c r="A46" s="15">
         <v>39</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F46" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G46" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H46" s="17" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="I46" s="17" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="J46" s="16" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K46" s="16">
         <v>15</v>
@@ -4216,46 +4181,46 @@
       <c r="L46" s="16"/>
       <c r="M46" s="16"/>
     </row>
-    <row r="47" spans="1:13" ht="82.5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" ht="66">
       <c r="A47" s="10">
         <v>40</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="D47" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="E47" s="14" t="s">
-        <v>13</v>
-      </c>
       <c r="F47" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G47" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H47" s="13" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="I47" s="13" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="J47" s="11" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K47" s="11">
         <v>40</v>
       </c>
       <c r="L47" s="11" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="M47" s="11"/>
     </row>
-    <row r="48" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" ht="16.5">
       <c r="A48" s="15"/>
       <c r="B48" s="6"/>
       <c r="C48" s="7"/>
@@ -4272,36 +4237,36 @@
       <c r="L48" s="16"/>
       <c r="M48" s="16"/>
     </row>
-    <row r="49" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" ht="33">
       <c r="A49" s="15">
         <v>41</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D49" s="18" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E49" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F49" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G49" s="16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H49" s="17" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="I49" s="17" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="J49" s="16" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K49" s="16">
         <v>35</v>
@@ -4309,75 +4274,75 @@
       <c r="L49" s="16"/>
       <c r="M49" s="16"/>
     </row>
-    <row r="50" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" ht="33">
       <c r="A50" s="10">
         <v>42</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F50" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G50" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H50" s="13" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="I50" s="13" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="J50" s="11" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K50" s="11">
         <v>30</v>
       </c>
       <c r="L50" s="11"/>
       <c r="M50" s="11" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="51" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" ht="33">
       <c r="A51" s="10">
         <v>43</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G51" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H51" s="13" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="I51" s="13" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="J51" s="11" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K51" s="11">
         <v>35</v>
@@ -4385,36 +4350,36 @@
       <c r="L51" s="11"/>
       <c r="M51" s="11"/>
     </row>
-    <row r="52" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13" ht="49.5">
       <c r="A52" s="15">
         <v>44</v>
       </c>
       <c r="B52" s="16" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C52" s="18" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D52" s="7" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="E52" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F52" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G52" s="16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H52" s="17" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="I52" s="17" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="J52" s="16" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K52" s="16">
         <v>35</v>
@@ -4422,36 +4387,36 @@
       <c r="L52" s="16"/>
       <c r="M52" s="16"/>
     </row>
-    <row r="53" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:13" ht="33">
       <c r="A53" s="15">
         <v>45</v>
       </c>
       <c r="B53" s="16" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C53" s="18" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E53" s="18" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F53" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G53" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H53" s="17" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="I53" s="17" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="J53" s="16" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K53" s="16">
         <v>15</v>
@@ -4459,36 +4424,36 @@
       <c r="L53" s="16"/>
       <c r="M53" s="16"/>
     </row>
-    <row r="54" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:13" ht="33">
       <c r="A54" s="15">
         <v>46</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="D54" s="7" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F54" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G54" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H54" s="17" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="I54" s="17" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="J54" s="16" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K54" s="16">
         <v>35</v>
@@ -4496,36 +4461,36 @@
       <c r="L54" s="16"/>
       <c r="M54" s="16"/>
     </row>
-    <row r="55" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13" ht="33">
       <c r="A55" s="15">
         <v>47</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F55" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H55" s="17" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="I55" s="17" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="J55" s="16" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K55" s="16">
         <v>40</v>
@@ -4533,7 +4498,7 @@
       <c r="L55" s="16"/>
       <c r="M55" s="16"/>
     </row>
-    <row r="56" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:13" ht="16.5">
       <c r="A56" s="15"/>
       <c r="B56" s="6"/>
       <c r="C56" s="7"/>
@@ -4550,75 +4515,75 @@
       <c r="L56" s="16"/>
       <c r="M56" s="16"/>
     </row>
-    <row r="57" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:13" ht="33">
       <c r="A57" s="10">
         <v>48</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="D57" s="14" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="E57" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G57" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H57" s="13" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="I57" s="13" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K57" s="11">
         <v>35</v>
       </c>
       <c r="L57" s="11"/>
       <c r="M57" s="11" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="58" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" ht="49.5">
       <c r="A58" s="10">
         <v>49</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="D58" s="14" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E58" s="14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G58" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H58" s="13" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="I58" s="13" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="J58" s="11" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K58" s="11">
         <v>15</v>
@@ -4626,36 +4591,36 @@
       <c r="L58" s="11"/>
       <c r="M58" s="11"/>
     </row>
-    <row r="59" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13" ht="49.5">
       <c r="A59" s="10">
         <v>50</v>
       </c>
       <c r="B59" s="20" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G59" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H59" s="13" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="I59" s="13" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="J59" s="11" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K59" s="11">
         <v>40</v>
@@ -4663,36 +4628,36 @@
       <c r="L59" s="11"/>
       <c r="M59" s="11"/>
     </row>
-    <row r="60" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:13" ht="33">
       <c r="A60" s="10">
         <v>51</v>
       </c>
       <c r="B60" s="20" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C60" s="12" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G60" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H60" s="13" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="I60" s="13" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="J60" s="11" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K60" s="11">
         <v>40</v>
@@ -4700,7 +4665,7 @@
       <c r="L60" s="11"/>
       <c r="M60" s="11"/>
     </row>
-    <row r="61" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:13" ht="16.5">
       <c r="A61" s="15"/>
       <c r="B61" s="6"/>
       <c r="C61" s="7"/>
@@ -4717,36 +4682,36 @@
       <c r="L61" s="16"/>
       <c r="M61" s="16"/>
     </row>
-    <row r="62" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:13" ht="16.5">
       <c r="A62" s="15">
         <v>52</v>
       </c>
       <c r="B62" s="16" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C62" s="18" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="D62" s="18" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="E62" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F62" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G62" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H62" s="17" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="I62" s="17" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="J62" s="16" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K62" s="16">
         <v>35</v>
@@ -4754,7 +4719,7 @@
       <c r="L62" s="16"/>
       <c r="M62" s="16"/>
     </row>
-    <row r="63" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:13" ht="16.5">
       <c r="A63" s="15"/>
       <c r="B63" s="6"/>
       <c r="C63" s="7"/>
@@ -4771,36 +4736,36 @@
       <c r="L63" s="16"/>
       <c r="M63" s="16"/>
     </row>
-    <row r="64" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:13" ht="47.25">
       <c r="A64" s="15">
         <v>53</v>
       </c>
       <c r="B64" s="22" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="C64" s="23" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="D64" s="7" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="E64" s="7" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F64" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G64" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H64" s="17" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="I64" s="17" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="J64" s="16" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K64" s="16">
         <v>35</v>
@@ -4808,114 +4773,114 @@
       <c r="L64" s="16"/>
       <c r="M64" s="16"/>
     </row>
-    <row r="65" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" ht="33">
       <c r="A65" s="15">
         <v>54</v>
       </c>
       <c r="B65" s="16" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="C65" s="18" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="D65" s="18" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E65" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F65" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G65" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H65" s="17" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="I65" s="17" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="J65" s="16" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K65" s="16">
         <v>30</v>
       </c>
       <c r="L65" s="16"/>
       <c r="M65" s="16" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="66" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" ht="33">
       <c r="A66" s="10">
         <v>55</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="C66" s="12" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="D66" s="12" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="E66" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G66" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H66" s="13" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="I66" s="13" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="J66" s="11" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K66" s="11">
         <v>30</v>
       </c>
       <c r="L66" s="11"/>
       <c r="M66" s="11" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="67" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" ht="33">
       <c r="A67" s="10">
         <v>56</v>
       </c>
       <c r="B67" s="20" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="D67" s="12" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E67" s="12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G67" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H67" s="13" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="I67" s="13" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="J67" s="11" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K67" s="11">
         <v>15</v>
@@ -4923,36 +4888,36 @@
       <c r="L67" s="11"/>
       <c r="M67" s="11"/>
     </row>
-    <row r="68" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" ht="33">
       <c r="A68" s="10">
         <v>57</v>
       </c>
       <c r="B68" s="20" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="D68" s="12" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E68" s="12" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F68" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G68" s="11" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H68" s="13" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="I68" s="13" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="J68" s="11" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K68" s="11">
         <v>20</v>
@@ -4960,36 +4925,36 @@
       <c r="L68" s="11"/>
       <c r="M68" s="11"/>
     </row>
-    <row r="69" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" ht="49.5">
       <c r="A69" s="15">
         <v>58</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="C69" s="18" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="E69" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F69" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G69" s="16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H69" s="17" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="I69" s="17" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J69" s="16" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K69" s="16">
         <v>35</v>
@@ -4997,36 +4962,36 @@
       <c r="L69" s="16"/>
       <c r="M69" s="16"/>
     </row>
-    <row r="70" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" ht="33">
       <c r="A70" s="15">
         <v>59</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="D70" s="7" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="E70" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F70" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G70" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H70" s="17" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="I70" s="17" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J70" s="16" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K70" s="16">
         <v>35</v>
@@ -5034,36 +4999,36 @@
       <c r="L70" s="16"/>
       <c r="M70" s="16"/>
     </row>
-    <row r="71" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" ht="33">
       <c r="A71" s="15">
         <v>60</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="E71" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F71" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G71" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H71" s="17" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="I71" s="17" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="J71" s="16" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K71" s="16">
         <v>40</v>
@@ -5071,7 +5036,7 @@
       <c r="L71" s="16"/>
       <c r="M71" s="16"/>
     </row>
-    <row r="72" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" ht="16.5">
       <c r="A72" s="15"/>
       <c r="B72" s="6"/>
       <c r="C72" s="7"/>
@@ -5088,75 +5053,75 @@
       <c r="L72" s="16"/>
       <c r="M72" s="16"/>
     </row>
-    <row r="73" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" ht="33">
       <c r="A73" s="15">
         <v>61</v>
       </c>
       <c r="B73" s="16" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="C73" s="18" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="D73" s="18" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="E73" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F73" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G73" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H73" s="17" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="I73" s="17" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="J73" s="16" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K73" s="16">
         <v>30</v>
       </c>
       <c r="L73" s="16"/>
       <c r="M73" s="16" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="74" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" ht="33">
       <c r="A74" s="15">
         <v>62</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="D74" s="7" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E74" s="7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F74" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G74" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H74" s="17" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="I74" s="17" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="J74" s="16" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K74" s="16">
         <v>15</v>
@@ -5164,36 +5129,36 @@
       <c r="L74" s="16"/>
       <c r="M74" s="16"/>
     </row>
-    <row r="75" spans="1:13" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" ht="47.25">
       <c r="A75" s="15">
         <v>63</v>
       </c>
       <c r="B75" s="22" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="C75" s="23" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="E75" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F75" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G75" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H75" s="17" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="I75" s="17" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="J75" s="16" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K75" s="16">
         <v>35</v>
@@ -5201,27 +5166,27 @@
       <c r="L75" s="16"/>
       <c r="M75" s="16"/>
     </row>
-    <row r="76" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" ht="49.5">
       <c r="A76" s="10">
         <v>64</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D76" s="12" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="E76" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F76" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G76" s="11" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H76" s="19">
         <v>46062</v>
@@ -5230,7 +5195,7 @@
         <v>46066</v>
       </c>
       <c r="J76" s="11" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K76" s="11">
         <v>35</v>
@@ -5238,27 +5203,27 @@
       <c r="L76" s="11"/>
       <c r="M76" s="11"/>
     </row>
-    <row r="77" spans="1:13" ht="66" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" ht="49.5">
       <c r="A77" s="10">
         <v>65</v>
       </c>
       <c r="B77" s="11" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="C77" s="12" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="D77" s="14" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E77" s="14" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="F77" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G77" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H77" s="19">
         <v>46062</v>
@@ -5267,7 +5232,7 @@
         <v>46066</v>
       </c>
       <c r="J77" s="11" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K77" s="11">
         <v>15</v>
@@ -5275,36 +5240,36 @@
       <c r="L77" s="11"/>
       <c r="M77" s="11"/>
     </row>
-    <row r="78" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" ht="33">
       <c r="A78" s="10">
         <v>66</v>
       </c>
       <c r="B78" s="20" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="C78" s="12" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="D78" s="14" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="E78" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F78" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G78" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H78" s="13" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="I78" s="13" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="J78" s="11" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K78" s="11">
         <v>35</v>
@@ -5312,36 +5277,36 @@
       <c r="L78" s="11"/>
       <c r="M78" s="11"/>
     </row>
-    <row r="79" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" ht="33">
       <c r="A79" s="10">
         <v>67</v>
       </c>
       <c r="B79" s="20" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="D79" s="12" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E79" s="12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F79" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G79" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H79" s="13" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="I79" s="13" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="J79" s="11" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K79" s="11">
         <v>15</v>
@@ -5349,36 +5314,36 @@
       <c r="L79" s="11"/>
       <c r="M79" s="11"/>
     </row>
-    <row r="80" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" ht="33">
       <c r="A80" s="15">
         <v>68</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="D80" s="7" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E80" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F80" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G80" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H80" s="17" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="I80" s="17" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="J80" s="16" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K80" s="16">
         <v>35</v>
@@ -5386,36 +5351,36 @@
       <c r="L80" s="16"/>
       <c r="M80" s="16"/>
     </row>
-    <row r="81" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:13" ht="33">
       <c r="A81" s="15">
         <v>69</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="D81" s="7" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E81" s="7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F81" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G81" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H81" s="17" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="I81" s="17" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="J81" s="16" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K81" s="16">
         <v>15</v>
@@ -5423,36 +5388,36 @@
       <c r="L81" s="16"/>
       <c r="M81" s="16"/>
     </row>
-    <row r="82" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:13" ht="16.5">
       <c r="A82" s="10">
         <v>70</v>
       </c>
       <c r="B82" s="20" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="D82" s="14" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E82" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F82" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G82" s="11" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H82" s="13" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="I82" s="13" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="J82" s="11" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K82" s="11">
         <v>35</v>
@@ -5460,36 +5425,36 @@
       <c r="L82" s="11"/>
       <c r="M82" s="11"/>
     </row>
-    <row r="83" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:13" ht="33">
       <c r="A83" s="10">
         <v>71</v>
       </c>
       <c r="B83" s="20" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="C83" s="12" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="D83" s="12" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="E83" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F83" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G83" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H83" s="13" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="I83" s="13" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="J83" s="11" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K83" s="11">
         <v>35</v>
@@ -5497,36 +5462,36 @@
       <c r="L83" s="11"/>
       <c r="M83" s="11"/>
     </row>
-    <row r="84" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:13" ht="33">
       <c r="A84" s="10">
         <v>72</v>
       </c>
       <c r="B84" s="20" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="C84" s="12" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="D84" s="12" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E84" s="12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F84" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G84" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H84" s="13" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="I84" s="13" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="J84" s="11" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K84" s="11">
         <v>15</v>
@@ -5534,7 +5499,7 @@
       <c r="L84" s="11"/>
       <c r="M84" s="11"/>
     </row>
-    <row r="85" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:13" ht="16.5">
       <c r="A85" s="15"/>
       <c r="B85" s="6"/>
       <c r="C85" s="7"/>
@@ -5551,36 +5516,36 @@
       <c r="L85" s="16"/>
       <c r="M85" s="16"/>
     </row>
-    <row r="86" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:13" ht="33">
       <c r="A86" s="10">
         <v>73</v>
       </c>
       <c r="B86" s="20" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="C86" s="12" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="D86" s="12" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E86" s="12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F86" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G86" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H86" s="13" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="I86" s="13" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="J86" s="11" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K86" s="11">
         <v>15</v>
@@ -5588,36 +5553,36 @@
       <c r="L86" s="11"/>
       <c r="M86" s="11"/>
     </row>
-    <row r="87" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:13" ht="33">
       <c r="A87" s="10">
         <v>74</v>
       </c>
       <c r="B87" s="20" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="C87" s="12" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="D87" s="12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E87" s="12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F87" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G87" s="11" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H87" s="13" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="I87" s="13" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="J87" s="11" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K87" s="11">
         <v>15</v>
@@ -5625,36 +5590,36 @@
       <c r="L87" s="11"/>
       <c r="M87" s="11"/>
     </row>
-    <row r="88" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:13" ht="33">
       <c r="A88" s="10">
         <v>75</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="C88" s="14" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="D88" s="14" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="E88" s="14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F88" s="11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G88" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H88" s="13" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="I88" s="13" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="J88" s="11" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K88" s="11">
         <v>15</v>
@@ -5662,36 +5627,36 @@
       <c r="L88" s="11"/>
       <c r="M88" s="11"/>
     </row>
-    <row r="89" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:13" ht="33">
       <c r="A89" s="10">
         <v>76</v>
       </c>
       <c r="B89" s="20" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="D89" s="14" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="E89" s="12" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F89" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G89" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H89" s="13" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="I89" s="13" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="J89" s="11" t="s">
-        <v>33</v>
+        <v>290</v>
       </c>
       <c r="K89" s="11">
         <v>35</v>
@@ -5699,36 +5664,36 @@
       <c r="L89" s="11"/>
       <c r="M89" s="11"/>
     </row>
-    <row r="90" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:13" ht="49.5">
       <c r="A90" s="10">
         <v>77</v>
       </c>
       <c r="B90" s="20" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="C90" s="14" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D90" s="12" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="E90" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F90" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G90" s="11" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H90" s="13" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="I90" s="13" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="J90" s="11" t="s">
-        <v>18</v>
+        <v>288</v>
       </c>
       <c r="K90" s="11">
         <v>35</v>
@@ -5736,36 +5701,36 @@
       <c r="L90" s="11"/>
       <c r="M90" s="11"/>
     </row>
-    <row r="91" spans="1:13" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:13" ht="37.5">
       <c r="A91" s="15">
         <v>78</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="C91" s="24" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="D91" s="24" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="E91" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F91" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G91" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H91" s="17" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="I91" s="17" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="J91" s="16" t="s">
-        <v>29</v>
+        <v>289</v>
       </c>
       <c r="K91" s="16">
         <v>35</v>
@@ -5773,36 +5738,36 @@
       <c r="L91" s="16"/>
       <c r="M91" s="16"/>
     </row>
-    <row r="92" spans="1:13" ht="33" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:13" ht="33">
       <c r="A92" s="15">
         <v>79</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="D92" s="7" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="E92" s="7" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F92" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G92" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H92" s="17" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="I92" s="17" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="J92" s="16" t="s">
-        <v>85</v>
+        <v>291</v>
       </c>
       <c r="K92" s="16">
         <v>35</v>
@@ -5810,36 +5775,36 @@
       <c r="L92" s="16"/>
       <c r="M92" s="16"/>
     </row>
-    <row r="93" spans="1:13" ht="49.5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:13" ht="33">
       <c r="A93" s="10">
         <v>80</v>
       </c>
       <c r="B93" s="25" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="C93" s="26" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="D93" s="26" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="E93" s="26" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F93" s="27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G93" s="27" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H93" s="28" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="I93" s="28" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="J93" s="27" t="s">
-        <v>24</v>
+        <v>292</v>
       </c>
       <c r="K93" s="27">
         <v>40</v>
@@ -5847,7 +5812,7 @@
       <c r="L93" s="27"/>
       <c r="M93" s="27"/>
     </row>
-    <row r="94" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:13" ht="16.5">
       <c r="A94" s="34"/>
       <c r="B94" s="35"/>
       <c r="C94" s="36"/>
@@ -5875,43 +5840,43 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A63EB81-1118-4DA5-A249-9650BB50BE48}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="70.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="70.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="18.75">
       <c r="A1" s="46" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="B1" s="46"/>
       <c r="C1" s="46"/>
     </row>
-    <row r="2" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="18.75">
       <c r="A2" s="42" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="C2" s="45"/>
     </row>
-    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="18.75">
       <c r="A3" s="43"/>
       <c r="B3" s="38" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C3" s="38" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="18.75">
       <c r="A4" s="39" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="B4" s="39">
         <v>27</v>
@@ -5920,9 +5885,9 @@
         <v>940</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="18.75">
       <c r="A5" s="39" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="B5" s="39">
         <v>24</v>
@@ -5931,9 +5896,9 @@
         <v>890</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="18.75">
       <c r="A6" s="39" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="B6" s="39">
         <v>23</v>
@@ -5942,9 +5907,9 @@
         <v>345</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="18.75">
       <c r="A7" s="39" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="B7" s="39">
         <v>6</v>
@@ -5953,9 +5918,9 @@
         <v>140</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="18.75">
       <c r="A8" s="38" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="B8" s="38">
         <v>80</v>
@@ -5964,29 +5929,29 @@
         <v>2315</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="18.75">
       <c r="A10" s="41" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15.75">
       <c r="A11" s="40" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15.75">
       <c r="A12" s="40" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15.75">
       <c r="A13" s="40" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15.75">
       <c r="A14" s="40" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>